<commit_message>
feat: demo scenario v3 - manual upload, skill indicator, kanban board
依 docs/demo-scenario-v3.md 重做整個 demo 情境。

主要內容
- 開場改為手動把 Excel 拖進對話框，不再自動載入
- 呼吸燈顯示正在執行哪個 skill；沒有呼叫工具的回合不顯示運算字樣
- 司機規則一次問完三個參數（期限／單件重量／最晚收工），每個都附該車現況數字
- 新增第六種規則型別 LATEST_RETURN_TIME（最晚收工時間）
- 訂單看板改成四台車四欄，可跨車與同車拖曳、先試算再套用、上一步下一步
- 插單方案卡標明「責任區」或「跨區支援」
- 發車後調整新增「我自己排」，按下後自動捲到看板並鎖定已送達站點
- 成效回顧改為純文字，追問才出現套用卡片
- 未知訂單改回結構化 ORDER_NOT_FOUND，不再假成功

資料重產（我獨立量測確認）
  50 張訂單 → 50 個不同座標（原本 50 張只有 32 個座標）
  最近鄰距離 最小 605 m、中位數 900 m（原本中位數 0 m）
  小於 300 m 的點 0 個（原本 45 個）
  tight 49/50 229.1 km、relaxed 50/50 243.7 km

本輪修正
- 規則選項的最晚收工時間不再顯示成「目前 15:02 時間」，改為「目前 15:02」
  並補上「這台車目前最後一站預估 15:02 送達」

已知未解
- 單張急單目前只產生 1 張非支配方案卡（三張一起插為 2 張）

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/demo-50-guardrail-note.xlsx
+++ b/data/samples/demo-50-guardrail-note.xlsx
@@ -2,23 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet name="orders" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="packages" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="vehicles" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="zones" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'orders'!$A$1:$K$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'packages'!$A$1:$C$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'vehicles'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'zones'!$A$1:$I$6</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames/>
 </workbook>
 </file>
 
@@ -28,10 +18,8 @@
   <fonts count="1">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,24 +31,18 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -175,72 +157,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -296,7 +220,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -305,13 +229,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -345,17 +269,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -410,8 +323,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -424,7 +335,7 @@
   <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,24 +408,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>三重</t>
+          <t>北投</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-01</t>
+          <t>北投示範配送點 01</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>25.059348</v>
+        <v>25.126</v>
       </c>
       <c r="G2" t="n">
-        <v>121.487395</v>
+        <v>121.495</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -548,28 +459,28 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>板橋</t>
+          <t>北投</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-02</t>
+          <t>北投示範配送點 02</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.011579</v>
+        <v>25.132</v>
       </c>
       <c r="G3" t="n">
-        <v>121.458678</v>
+        <v>121.501</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -582,7 +493,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -599,28 +510,28 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>新莊</t>
+          <t>北投</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-03</t>
+          <t>北投示範配送點 03</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>25.033395</v>
+        <v>25.138</v>
       </c>
       <c r="G4" t="n">
-        <v>121.451894</v>
+        <v>121.507</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -633,7 +544,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -650,24 +561,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>新莊</t>
+          <t>士林</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-04</t>
+          <t>士林示範配送點 04</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>25.034619</v>
+        <v>25.087</v>
       </c>
       <c r="G5" t="n">
-        <v>121.449264</v>
+        <v>121.519</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -675,7 +586,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -684,7 +595,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -701,32 +612,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>三重</t>
+          <t>士林</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-05</t>
+          <t>士林示範配送點 05</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>25.060413</v>
+        <v>25.093</v>
       </c>
       <c r="G6" t="n">
-        <v>121.487777</v>
+        <v>121.525</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -735,7 +646,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -752,32 +663,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>新莊</t>
+          <t>士林</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-06</t>
+          <t>士林示範配送點 06</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>25.036783</v>
+        <v>25.099</v>
       </c>
       <c r="G7" t="n">
-        <v>121.452427</v>
+        <v>121.531</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -786,7 +697,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -803,24 +714,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>三重</t>
+          <t>大同</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-07</t>
+          <t>大同示範配送點 07</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>25.06389</v>
+        <v>25.057</v>
       </c>
       <c r="G8" t="n">
-        <v>121.485812</v>
+        <v>121.507</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -828,7 +739,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -837,7 +748,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -854,32 +765,32 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>新莊</t>
+          <t>大同</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-08</t>
+          <t>大同示範配送點 08</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>25.033948</v>
+        <v>25.063</v>
       </c>
       <c r="G9" t="n">
-        <v>121.45034</v>
+        <v>121.513</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -888,7 +799,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -905,32 +816,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>新莊</t>
+          <t>大同</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-09</t>
+          <t>大同示範配送點 09</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>25.033664</v>
+        <v>25.069</v>
       </c>
       <c r="G10" t="n">
-        <v>121.448133</v>
+        <v>121.519</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -939,7 +850,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -956,24 +867,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>三重</t>
+          <t>中山</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-10</t>
+          <t>中山示範配送點 10</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>25.060621</v>
+        <v>25.058</v>
       </c>
       <c r="G11" t="n">
-        <v>121.486005</v>
+        <v>121.527</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -981,7 +892,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -990,7 +901,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1007,32 +918,32 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>板橋</t>
+          <t>中山</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-11</t>
+          <t>中山示範配送點 11</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>25.01234</v>
+        <v>25.064</v>
       </c>
       <c r="G12" t="n">
-        <v>121.461405</v>
+        <v>121.533</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1041,7 +952,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1058,28 +969,28 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>板橋</t>
+          <t>中山</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>示範配送點 Z1-12</t>
+          <t>中山示範配送點 12</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>25.010355</v>
+        <v>25.07</v>
       </c>
       <c r="G13" t="n">
-        <v>121.461585</v>
+        <v>121.539</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1092,7 +1003,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1104,12 +1015,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1119,22 +1030,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-13</t>
+          <t>文山示範配送點 13</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>24.989312</v>
+        <v>24.983</v>
       </c>
       <c r="G14" t="n">
-        <v>121.568689</v>
+        <v>121.564</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1143,7 +1054,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1155,29 +1066,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>新店</t>
+          <t>大安</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-14</t>
+          <t>大安示範配送點 14</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>24.967468</v>
+        <v>25.02</v>
       </c>
       <c r="G15" t="n">
-        <v>121.544771</v>
+        <v>121.537</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1194,7 +1105,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1117,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1216,27 +1127,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>文山</t>
+          <t>中正</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-15</t>
+          <t>中正示範配送點 15</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>24.98912</v>
+        <v>25.026</v>
       </c>
       <c r="G16" t="n">
-        <v>121.571735</v>
+        <v>121.512</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1245,7 +1156,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1262,24 +1173,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>中和</t>
+          <t>南港</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-16</t>
+          <t>南港示範配送點 16</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>25.000834</v>
+        <v>25.049</v>
       </c>
       <c r="G17" t="n">
-        <v>121.495405</v>
+        <v>121.601</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1296,7 +1207,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1308,29 +1219,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>永和</t>
+          <t>萬華</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-17</t>
+          <t>萬華示範配送點 17</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>25.008146</v>
+        <v>25.022</v>
       </c>
       <c r="G18" t="n">
-        <v>121.512855</v>
+        <v>121.491</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1338,7 +1249,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1347,7 +1258,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1369,27 +1280,27 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>中和</t>
+          <t>南港</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-18</t>
+          <t>南港示範配送點 18</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>24.999782</v>
+        <v>25.055</v>
       </c>
       <c r="G19" t="n">
-        <v>121.498253</v>
+        <v>121.607</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1398,7 +1309,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1415,24 +1326,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>新店</t>
+          <t>松山</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-19</t>
+          <t>松山示範配送點 19</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>24.970087</v>
+        <v>25.052</v>
       </c>
       <c r="G20" t="n">
-        <v>121.541294</v>
+        <v>121.552</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1440,7 +1351,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1449,7 +1360,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1466,32 +1377,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>永和</t>
+          <t>內湖</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-20</t>
+          <t>內湖示範配送點 20</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>25.009453</v>
+        <v>25.063</v>
       </c>
       <c r="G21" t="n">
-        <v>121.512703</v>
+        <v>121.582</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1500,7 +1411,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1517,32 +1428,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>新店</t>
+          <t>南港</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-21</t>
+          <t>南港示範配送點 21</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>24.968948</v>
+        <v>25.061</v>
       </c>
       <c r="G22" t="n">
-        <v>121.540753</v>
+        <v>121.613</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1551,7 +1462,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1568,24 +1479,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>永和</t>
+          <t>松山</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-22</t>
+          <t>松山示範配送點 22</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>25.010902</v>
+        <v>25.058</v>
       </c>
       <c r="G23" t="n">
-        <v>121.516256</v>
+        <v>121.558</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1593,7 +1504,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1602,7 +1513,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1624,27 +1535,27 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>文山</t>
+          <t>信義</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>示範配送點 Z2-23</t>
+          <t>信義示範配送點 23</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>24.987875</v>
+        <v>25.027</v>
       </c>
       <c r="G24" t="n">
-        <v>121.569941</v>
+        <v>121.565</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1653,7 +1564,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1576,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1675,23 +1586,23 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>中山</t>
+          <t>信義</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-24</t>
+          <t>信義示範配送點 24</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>25.050494</v>
+        <v>25.039</v>
       </c>
       <c r="G25" t="n">
-        <v>121.530972</v>
+        <v>121.577</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -1704,7 +1615,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1726,23 +1637,23 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>中山</t>
+          <t>萬華</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-25</t>
+          <t>萬華示範配送點 25</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>25.053608</v>
+        <v>25.028</v>
       </c>
       <c r="G26" t="n">
-        <v>121.533295</v>
+        <v>121.497</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -1755,7 +1666,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1777,19 +1688,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>萬華</t>
+          <t>中正</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-26</t>
+          <t>中正示範配送點 26</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>25.033703</v>
+        <v>25.032</v>
       </c>
       <c r="G27" t="n">
-        <v>121.497945</v>
+        <v>121.518</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1806,7 +1717,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1828,27 +1739,27 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>中正</t>
+          <t>大安</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-27</t>
+          <t>大安示範配送點 27</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>25.031881</v>
+        <v>25.026</v>
       </c>
       <c r="G28" t="n">
-        <v>121.51809</v>
+        <v>121.543</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1857,7 +1768,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1879,27 +1790,27 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>大同</t>
+          <t>文山</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-28</t>
+          <t>文山示範配送點 28</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>25.064615</v>
+        <v>24.989</v>
       </c>
       <c r="G29" t="n">
-        <v>121.510607</v>
+        <v>121.57</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1908,7 +1819,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1930,19 +1841,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>中正</t>
+          <t>萬華</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-29</t>
+          <t>萬華示範配送點 29</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>25.034585</v>
+        <v>25.034</v>
       </c>
       <c r="G30" t="n">
-        <v>121.517571</v>
+        <v>121.503</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1950,7 +1861,7 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1959,7 +1870,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -1981,23 +1892,23 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>中山</t>
+          <t>中正</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-30</t>
+          <t>中正示範配送點 30</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>25.052987</v>
+        <v>25.038</v>
       </c>
       <c r="G31" t="n">
-        <v>121.534857</v>
+        <v>121.524</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -2010,7 +1921,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2032,27 +1943,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>萬華</t>
+          <t>大安</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-31</t>
+          <t>大安示範配送點 31</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>25.034205</v>
+        <v>25.032</v>
       </c>
       <c r="G32" t="n">
-        <v>121.499354</v>
+        <v>121.549</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2061,7 +1972,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2073,37 +1984,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Z3</t>
+          <t>Z5</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>中正</t>
+          <t>新店</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-32</t>
+          <t>新店示範配送點 32</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>25.033932</v>
+        <v>24.961</v>
       </c>
       <c r="G33" t="n">
-        <v>121.521396</v>
+        <v>121.535</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>EVENING</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2112,7 +2023,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2134,27 +2045,27 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>中山</t>
+          <t>文山</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>示範配送點 Z3-33</t>
+          <t>文山示範配送點 33</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>25.050736</v>
+        <v>24.995</v>
       </c>
       <c r="G34" t="n">
-        <v>121.535548</v>
+        <v>121.576</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2163,7 +2074,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2180,32 +2091,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>大安</t>
+          <t>板橋</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-34</t>
+          <t>板橋示範配送點 34</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>25.025333</v>
+        <v>25.005</v>
       </c>
       <c r="G35" t="n">
-        <v>121.542809</v>
+        <v>121.453</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2214,7 +2125,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2231,24 +2142,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>南港</t>
+          <t>板橋</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-35</t>
+          <t>板橋示範配送點 35</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>25.053403</v>
+        <v>25.017</v>
       </c>
       <c r="G36" t="n">
-        <v>121.603725</v>
+        <v>121.465</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2256,7 +2167,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2265,7 +2176,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2282,32 +2193,32 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>大安</t>
+          <t>新莊</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-36</t>
+          <t>新莊示範配送點 36</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>25.027962</v>
+        <v>25.03</v>
       </c>
       <c r="G37" t="n">
-        <v>121.542175</v>
+        <v>121.444</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2316,7 +2227,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2239,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Z4</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2338,19 +2249,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>松山</t>
+          <t>內湖</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-37</t>
+          <t>內湖示範配送點 37</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>25.049652</v>
+        <v>25.075</v>
       </c>
       <c r="G38" t="n">
-        <v>121.556441</v>
+        <v>121.594</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2358,7 +2269,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2367,7 +2278,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2384,24 +2295,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>南港</t>
+          <t>新莊</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-38</t>
+          <t>新莊示範配送點 38</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>25.053245</v>
+        <v>25.042</v>
       </c>
       <c r="G39" t="n">
-        <v>121.608648</v>
+        <v>121.456</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2409,7 +2320,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2418,7 +2329,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2435,28 +2346,28 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>大安</t>
+          <t>三重</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-39</t>
+          <t>三重示範配送點 39</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>25.026135</v>
+        <v>25.055</v>
       </c>
       <c r="G40" t="n">
-        <v>121.544154</v>
+        <v>121.481</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -2469,7 +2380,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2486,32 +2397,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>南港</t>
+          <t>三重</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-40</t>
+          <t>三重示範配送點 40</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>25.056813</v>
+        <v>25.067</v>
       </c>
       <c r="G41" t="n">
-        <v>121.609988</v>
+        <v>121.493</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2520,7 +2431,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2537,24 +2448,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>松山</t>
+          <t>蘆洲</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-41</t>
+          <t>蘆洲示範配送點 41</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>25.047981</v>
+        <v>25.079</v>
       </c>
       <c r="G42" t="n">
-        <v>121.558643</v>
+        <v>121.467</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2571,7 +2482,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2494,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Z4</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2593,23 +2504,23 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>信義</t>
+          <t>松山</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>示範配送點 Z4-42</t>
+          <t>松山示範配送點 42</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>25.032707</v>
+        <v>25.064</v>
       </c>
       <c r="G43" t="n">
-        <v>121.562765</v>
+        <v>121.564</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>EVENING</t>
+          <t>MORNING</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -2622,7 +2533,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2634,46 +2545,46 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Z5</t>
+          <t>Z4</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>內湖</t>
+          <t>蘆洲</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-43</t>
+          <t>蘆洲示範配送點 43</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>25.08121</v>
+        <v>25.091</v>
       </c>
       <c r="G44" t="n">
-        <v>121.590249</v>
+        <v>121.479</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>AFTERNOON</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>NORMAL</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2690,32 +2601,32 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>內湖</t>
+          <t>中和</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-44</t>
+          <t>中和示範配送點 44</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>25.084976</v>
+        <v>24.993</v>
       </c>
       <c r="G45" t="n">
-        <v>121.591166</v>
+        <v>121.492</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>EVENING</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -2724,7 +2635,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2741,24 +2652,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>北投</t>
+          <t>中和</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-45</t>
+          <t>中和示範配送點 45</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>25.133873</v>
+        <v>25.005</v>
       </c>
       <c r="G46" t="n">
-        <v>121.50187</v>
+        <v>121.504</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2766,7 +2677,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -2775,7 +2686,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2792,32 +2703,32 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>北投</t>
+          <t>永和</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-46</t>
+          <t>永和示範配送點 46</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>25.132546</v>
+        <v>25.002</v>
       </c>
       <c r="G47" t="n">
-        <v>121.503765</v>
+        <v>121.509</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>EVENING</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -2826,7 +2737,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2843,32 +2754,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>士林</t>
+          <t>永和</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-47</t>
+          <t>永和示範配送點 47</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>25.095239</v>
+        <v>25.014</v>
       </c>
       <c r="G48" t="n">
-        <v>121.522636</v>
+        <v>121.521</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>EVENING</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2877,7 +2788,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2894,24 +2805,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>內湖</t>
+          <t>土城</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-48</t>
+          <t>土城示範配送點 48</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>25.085241</v>
+        <v>24.966</v>
       </c>
       <c r="G49" t="n">
-        <v>121.593305</v>
+        <v>121.437</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2919,7 +2830,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -2928,7 +2839,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2945,32 +2856,32 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>士林</t>
+          <t>土城</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-49</t>
+          <t>土城示範配送點 49</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>25.094228</v>
+        <v>24.978</v>
       </c>
       <c r="G50" t="n">
-        <v>121.528385</v>
+        <v>121.449</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>MORNING</t>
+          <t>EVENING</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2979,7 +2890,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
@@ -2996,28 +2907,28 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>北投</t>
+          <t>新店</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>示範配送點 Z5-50</t>
+          <t>新店示範配送點 50</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>25.131841</v>
+        <v>24.973</v>
       </c>
       <c r="G51" t="n">
-        <v>121.50185</v>
+        <v>121.547</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>AFTERNOON</t>
+          <t>EVENING</t>
         </is>
       </c>
       <c r="I51" t="n">
@@ -3030,13 +2941,12 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>seed=260905; synthetic v2 demo fixture</t>
+          <t>seed=260905; synthetic v3 demo fixture</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K51"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -3049,7 +2959,7 @@
   <dimension ref="A1:C100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3081,7 +2991,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="3">
@@ -3096,7 +3006,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="4">
@@ -3111,7 +3021,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="5">
@@ -3126,7 +3036,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="6">
@@ -3141,7 +3051,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="7">
@@ -3156,28 +3066,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5.7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PKG-005-01</t>
+          <t>PKG-004-02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ORD-005</t>
+          <t>ORD-004</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PKG-005-02</t>
+          <t>PKG-005-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3186,13 +3096,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PKG-005-03</t>
+          <t>PKG-005-02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3201,7 +3111,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.3</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="11">
@@ -3216,28 +3126,28 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PKG-007-01</t>
+          <t>PKG-006-02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ORD-007</t>
+          <t>ORD-006</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PKG-007-02</t>
+          <t>PKG-007-01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3246,13 +3156,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PKG-007-03</t>
+          <t>PKG-007-02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3261,7 +3171,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="15">
@@ -3276,28 +3186,28 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7.5</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PKG-009-01</t>
+          <t>PKG-008-02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORD-009</t>
+          <t>ORD-008</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PKG-009-02</t>
+          <t>PKG-009-01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3306,13 +3216,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PKG-009-03</t>
+          <t>PKG-009-02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3321,7 +3231,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="19">
@@ -3336,28 +3246,28 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PKG-011-01</t>
+          <t>PKG-010-02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ORD-011</t>
+          <t>ORD-010</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PKG-011-02</t>
+          <t>PKG-011-01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3366,13 +3276,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PKG-011-03</t>
+          <t>PKG-011-02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3381,7 +3291,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="23">
@@ -3396,7 +3306,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="24">
@@ -3411,7 +3321,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="25">
@@ -3426,28 +3336,28 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PKG-014-01</t>
+          <t>PKG-013-02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ORD-014</t>
+          <t>ORD-013</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PKG-014-02</t>
+          <t>PKG-014-01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3456,28 +3366,28 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PKG-015-01</t>
+          <t>PKG-014-02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ORD-015</t>
+          <t>ORD-014</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2.1</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PKG-015-02</t>
+          <t>PKG-015-01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3486,13 +3396,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PKG-015-03</t>
+          <t>PKG-015-02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3501,7 +3411,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="31">
@@ -3516,7 +3426,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32">
@@ -3531,7 +3441,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -3546,28 +3456,28 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PKG-018-01</t>
+          <t>PKG-017-02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ORD-018</t>
+          <t>ORD-017</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PKG-018-02</t>
+          <t>PKG-018-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3576,13 +3486,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PKG-018-03</t>
+          <t>PKG-018-02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3591,7 +3501,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
@@ -3606,28 +3516,28 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PKG-020-01</t>
+          <t>PKG-019-02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ORD-020</t>
+          <t>ORD-019</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PKG-020-02</t>
+          <t>PKG-020-01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3636,13 +3546,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PKG-020-03</t>
+          <t>PKG-020-02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3651,7 +3561,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
@@ -3666,7 +3576,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -3681,28 +3591,28 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PKG-021-03</t>
+          <t>PKG-022-01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ORD-021</t>
+          <t>ORD-022</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PKG-022-01</t>
+          <t>PKG-022-02</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3711,7 +3621,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -3726,28 +3636,28 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PKG-024-01</t>
+          <t>PKG-023-02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ORD-024</t>
+          <t>ORD-023</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PKG-024-02</t>
+          <t>PKG-024-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3756,28 +3666,28 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PKG-025-01</t>
+          <t>PKG-024-02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ORD-025</t>
+          <t>ORD-024</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PKG-025-02</t>
+          <t>PKG-025-01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3786,28 +3696,28 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>5.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PKG-026-01</t>
+          <t>PKG-025-02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ORD-026</t>
+          <t>ORD-025</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PKG-026-02</t>
+          <t>PKG-026-01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3816,513 +3726,513 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PKG-027-01</t>
+          <t>PKG-026-02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ORD-027</t>
+          <t>ORD-026</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>5.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PKG-028-01</t>
+          <t>PKG-027-01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ORD-028</t>
+          <t>ORD-027</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>7.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PKG-029-01</t>
+          <t>PKG-027-02</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ORD-029</t>
+          <t>ORD-027</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>5.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PKG-030-01</t>
+          <t>PKG-028-01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ORD-030</t>
+          <t>ORD-028</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PKG-030-02</t>
+          <t>PKG-028-02</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ORD-030</t>
+          <t>ORD-028</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PKG-031-01</t>
+          <t>PKG-029-01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ORD-031</t>
+          <t>ORD-029</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PKG-031-02</t>
+          <t>PKG-029-02</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ORD-031</t>
+          <t>ORD-029</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PKG-031-03</t>
+          <t>PKG-030-01</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ORD-031</t>
+          <t>ORD-030</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PKG-032-01</t>
+          <t>PKG-030-02</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ORD-032</t>
+          <t>ORD-030</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>5.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PKG-033-01</t>
+          <t>PKG-031-01</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ORD-033</t>
+          <t>ORD-031</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>5.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PKG-034-01</t>
+          <t>PKG-031-02</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ORD-034</t>
+          <t>ORD-031</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2.1</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>PKG-034-02</t>
+          <t>PKG-032-01</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ORD-034</t>
+          <t>ORD-032</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3.9</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PKG-034-03</t>
+          <t>PKG-032-02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ORD-034</t>
+          <t>ORD-032</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PKG-035-01</t>
+          <t>PKG-033-01</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ORD-035</t>
+          <t>ORD-033</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PKG-035-02</t>
+          <t>PKG-033-02</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ORD-035</t>
+          <t>ORD-033</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PKG-035-03</t>
+          <t>PKG-034-01</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ORD-035</t>
+          <t>ORD-034</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PKG-036-01</t>
+          <t>PKG-034-02</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ORD-036</t>
+          <t>ORD-034</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>6.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>PKG-037-01</t>
+          <t>PKG-035-01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ORD-037</t>
+          <t>ORD-035</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>PKG-037-02</t>
+          <t>PKG-035-02</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ORD-037</t>
+          <t>ORD-035</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>PKG-037-03</t>
+          <t>PKG-036-01</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ORD-037</t>
+          <t>ORD-036</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PKG-038-01</t>
+          <t>PKG-036-02</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ORD-038</t>
+          <t>ORD-036</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5.7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PKG-039-01</t>
+          <t>PKG-037-01</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ORD-039</t>
+          <t>ORD-037</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1.4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PKG-039-02</t>
+          <t>PKG-037-02</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ORD-039</t>
+          <t>ORD-037</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>PKG-040-01</t>
+          <t>PKG-038-01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ORD-040</t>
+          <t>ORD-038</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PKG-040-02</t>
+          <t>PKG-038-02</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ORD-040</t>
+          <t>ORD-038</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PKG-040-03</t>
+          <t>PKG-039-01</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ORD-040</t>
+          <t>ORD-039</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PKG-041-01</t>
+          <t>PKG-039-02</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ORD-041</t>
+          <t>ORD-039</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PKG-041-02</t>
+          <t>PKG-040-01</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ORD-041</t>
+          <t>ORD-040</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PKG-042-01</t>
+          <t>PKG-040-02</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ORD-042</t>
+          <t>ORD-040</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PKG-042-02</t>
+          <t>PKG-041-01</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ORD-042</t>
+          <t>ORD-041</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PKG-043-01</t>
+          <t>PKG-041-02</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ORD-043</t>
+          <t>ORD-041</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PKG-043-02</t>
+          <t>PKG-042-01</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ORD-043</t>
+          <t>ORD-042</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PKG-043-03</t>
+          <t>PKG-042-02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ORD-043</t>
+          <t>ORD-042</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PKG-044-01</t>
+          <t>PKG-043-01</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ORD-044</t>
+          <t>ORD-043</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -4332,22 +4242,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PKG-044-02</t>
+          <t>PKG-043-02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ORD-044</t>
+          <t>ORD-043</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PKG-044-03</t>
+          <t>PKG-044-01</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4356,28 +4266,28 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PKG-045-01</t>
+          <t>PKG-044-02</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ORD-045</t>
+          <t>ORD-044</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PKG-045-02</t>
+          <t>PKG-045-01</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4386,13 +4296,13 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PKG-045-03</t>
+          <t>PKG-045-02</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4401,7 +4311,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="91">
@@ -4416,7 +4326,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="92">
@@ -4431,28 +4341,28 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PKG-046-03</t>
+          <t>PKG-047-01</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ORD-046</t>
+          <t>ORD-047</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>4.6</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PKG-047-01</t>
+          <t>PKG-047-02</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4461,7 +4371,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="95">
@@ -4476,28 +4386,28 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PKG-049-01</t>
+          <t>PKG-048-02</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ORD-049</t>
+          <t>ORD-048</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PKG-049-02</t>
+          <t>PKG-049-01</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4506,13 +4416,13 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PKG-049-03</t>
+          <t>PKG-049-02</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4521,7 +4431,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="99">
@@ -4536,7 +4446,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>3.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="100">
@@ -4551,12 +4461,11 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C100"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4569,7 +4478,7 @@
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4633,7 +4542,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Z1|Z2|Z3</t>
+          <t>Z3|Z4|Z5</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4648,7 +4557,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Z1、Z2、Z3 可服務</t>
+          <t>西區、南區主責；中區備援車</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4580,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Z1|Z3|Z4</t>
+          <t>Z2|Z3|Z4|Z5</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4686,7 +4595,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Z4 東區路線示範車</t>
+          <t>中區主責；東區規則重排第二備援；西區與南區備援車</t>
         </is>
       </c>
     </row>
@@ -4705,11 +4614,11 @@
         <v>160</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Z2|Z4|Z5</t>
+          <t>Z1|Z2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4724,7 +4633,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Z4、Z5 長距離路線示範車</t>
+          <t>東區主責；北區備援車</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4656,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Z1|Z2|Z5</t>
+          <t>Z1|Z2|Z3</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4762,13 +4671,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Z5 北區路線示範車</t>
+          <t>北區主責；東區與中區相鄰備援車</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4781,7 +4689,7 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4839,28 +4747,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>新北西區</t>
+          <t>北區</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>新北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>板橋|新莊|三重</t>
+          <t>北投|士林|大同|中山</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>25.0114</v>
+        <v>25.088</v>
       </c>
       <c r="F2" t="n">
-        <v>121.4618</v>
+        <v>121.518</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NWT</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -4880,33 +4788,33 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>雙和文山</t>
+          <t>東區</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>新北市|臺北市</t>
+          <t>臺北市</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>中和|永和|新店|文山</t>
+          <t>內湖|南港|松山|信義</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>24.999</v>
+        <v>25.05375</v>
       </c>
       <c r="F3" t="n">
-        <v>121.498</v>
+        <v>121.581</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>NWT|TPE</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Z1|Z3|Z4</t>
+          <t>Z1|Z3</t>
         </is>
       </c>
       <c r="I3" t="b">
@@ -4921,7 +4829,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>臺北西北核心</t>
+          <t>中區</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4931,14 +4839,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>萬華|中正|大同|中山</t>
+          <t>萬華|中正|大安|信義|文山</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>25.033</v>
+        <v>25.0216</v>
       </c>
       <c r="F4" t="n">
-        <v>121.499</v>
+        <v>121.5398</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -4947,7 +4855,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Z1|Z2|Z4|Z5</t>
+          <t>Z2|Z4|Z5</t>
         </is>
       </c>
       <c r="I4" t="b">
@@ -4962,33 +4870,33 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>臺北核心東區</t>
+          <t>西區</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>大安|信義|松山|南港</t>
+          <t>三重|新莊|板橋|蘆洲</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>25.0268</v>
+        <v>25.04825</v>
       </c>
       <c r="F5" t="n">
-        <v>121.5434</v>
+        <v>121.46725</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>NWT</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Z2|Z3|Z5</t>
+          <t>Z1|Z5</t>
         </is>
       </c>
       <c r="I5" t="b">
@@ -5003,28 +4911,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>臺北北區</t>
+          <t>南區</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>臺北市</t>
+          <t>新北市|臺北市</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>士林|北投|內湖</t>
+          <t>中和|永和|土城|新店|文山</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>25.095</v>
+        <v>24.987</v>
       </c>
       <c r="F6" t="n">
-        <v>121.525</v>
+        <v>121.5134</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>NWT|TPE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -5037,7 +4945,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>